<commit_message>
29/05/2025 - Hoan thien not Logic
</commit_message>
<xml_diff>
--- a/Logical Design.xlsx
+++ b/Logical Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\One_Times\College\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B39BBC-C7AE-4E4D-BFD0-23CD35AB7F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A782496-B2C0-4985-8B64-BB3859AAA688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CB452E84-88D2-41ED-B9FE-3951C5FD72F9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <r>
       <t xml:space="preserve">3. Add thành viên vào Project:
@@ -497,6 +497,9 @@
   </si>
   <si>
     <t>Đang check dup như nào</t>
+  </si>
+  <si>
+    <t>Phần UI: thêm label cho các Subtask: Quá hạn, sắp đến hạn, hoàn thành</t>
   </si>
 </sst>
 </file>
@@ -1021,6 +1024,9 @@
       <c r="B18" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="C18" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B20" s="7" t="s">

</xml_diff>

<commit_message>
01/06/2025 - commit truoc khi viet hoa toan bo project
</commit_message>
<xml_diff>
--- a/Logical Design.xlsx
+++ b/Logical Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\One_Times\College\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A782496-B2C0-4985-8B64-BB3859AAA688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{131D5339-650E-49D6-A176-7A3D178260E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CB452E84-88D2-41ED-B9FE-3951C5FD72F9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <r>
       <t xml:space="preserve">3. Add thành viên vào Project:
@@ -500,6 +500,54 @@
   </si>
   <si>
     <t>Phần UI: thêm label cho các Subtask: Quá hạn, sắp đến hạn, hoàn thành</t>
+  </si>
+  <si>
+    <t>DASHBOARD</t>
+  </si>
+  <si>
+    <t>1. Dự án gần đây</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Lấy 3 dự án được cập nhật gần đây nhất</t>
+  </si>
+  <si>
+    <t>2. Deadline sắp tới</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Top 5 tasks/projects có deadline gần nhất</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Tiêu chí sắp xếp: Ngày hết hạn tăng dần</t>
+  </si>
+  <si>
+    <t>3. Phân tích hiệu suất</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.1 Workload </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Đo lường mức độ bận rộn của nhân viên: (In Progress Tasks + Overdue Tasks) / Total Assigned Tasks × 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.2 Tỷ lệ hoàn thành đúng hạn </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - On-time Rate = Số task hoàn thành đúng/sớm hạn / Tổng số task đã hoàn thành × 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Điều kiện đúng hạn: lastModifiedDate ≤ dueDate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.3 Thời gian hoàn thành trung bình </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Average Days = Σ(lastModifiedDate - startDate) / Số task đã hoàn thành</t>
+  </si>
+  <si>
+    <t>3.4 Điểm hiệu suất tổng hợp</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Performance Score = (Completion Rate × 40% + On-time Rate × 35% + Consistency Score × 25%) × 100</t>
   </si>
 </sst>
 </file>
@@ -586,7 +634,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -614,6 +662,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -930,7 +981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CACC56E-65EC-46F3-A431-6E5D31AE7C57}">
-  <dimension ref="B1:C24"/>
+  <dimension ref="B1:C41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -1054,6 +1105,86 @@
     <row r="24" spans="2:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B24" s="2" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B26" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B27" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B28" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B29" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B30" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B31" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B32" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B33" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B36" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B37" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B38" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B39" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B40" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B41" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
01/06/2025 - Chính thức hoàn thành Web App Project Management Enter Track
</commit_message>
<xml_diff>
--- a/Logical Design.xlsx
+++ b/Logical Design.xlsx
@@ -8,15 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\One_Times\College\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{131D5339-650E-49D6-A176-7A3D178260E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E73851-2DB1-4BE1-874C-4A5072039988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CB452E84-88D2-41ED-B9FE-3951C5FD72F9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{CB452E84-88D2-41ED-B9FE-3951C5FD72F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Special" sheetId="1" r:id="rId1"/>
-    <sheet name="Add" sheetId="3" r:id="rId2"/>
-    <sheet name="Note" sheetId="2" r:id="rId3"/>
-    <sheet name="Ex" sheetId="4" r:id="rId4"/>
+    <sheet name="Ex" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <r>
       <t xml:space="preserve">3. Add thành viên vào Project:
@@ -342,9 +340,6 @@
 - Cập nhật trạng thái Proejct thành IN_PROGRESS nếu có ít nhất 1 Task chưa hoàn thành
 - Cập nhật trạng thái Task thành IN_PROGRESS nếu có ít nhất 1 Subtask chưa hoàn thành</t>
     </r>
-  </si>
-  <si>
-    <t>Người tạo task và subtask phải là PROJECT MANAGER</t>
   </si>
   <si>
     <t>1. Thêm tokenVersion  vào Users để viết hàm invalid user token để tận dụng cơ chế kiểm tra token hiện có để kích user ra ngoài</t>
@@ -634,7 +629,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -664,7 +659,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -985,7 +983,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="63.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="89.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48.109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="55.6640625" style="1" customWidth="1"/>
     <col min="5" max="16384" width="8.88671875" style="1"/>
@@ -996,14 +994,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="2:3" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" ht="72" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" s="10"/>
     </row>
@@ -1040,15 +1038,15 @@
     </row>
     <row r="11" spans="2:3" ht="72" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>20</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -1068,7 +1066,7 @@
     </row>
     <row r="17" spans="2:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B17" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="86.4" x14ac:dyDescent="0.3">
@@ -1076,7 +1074,7 @@
         <v>10</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
@@ -1089,7 +1087,7 @@
         <v>12</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="86.4" x14ac:dyDescent="0.3">
@@ -1109,82 +1107,82 @@
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B26" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B27" s="11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B27" s="1" t="s">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B28" s="12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B28" s="1" t="s">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B29" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B29" s="1" t="s">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B30" s="12" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B30" s="1" t="s">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B31" s="12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B31" s="1" t="s">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B32" s="11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B32" s="1" t="s">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B33" s="12" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B33" s="1" t="s">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" s="12" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B34" s="1" t="s">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" s="12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B35" s="1" t="s">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B36" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B36" s="1" t="s">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B37" s="12" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B37" s="1" t="s">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B38" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B38" s="1" t="s">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B39" s="12" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B39" s="1" t="s">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B40" s="12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B40" s="1" t="s">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B41" s="12" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B41" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1194,42 +1192,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC999140-D26F-4E3B-B27E-D592A400BAB6}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A1D2F6F-27B0-4203-938C-4728F3C6C1BA}">
-  <dimension ref="B11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4470116-0F26-4A65-970F-AC3E3EE82D95}">
   <dimension ref="B2:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>